<commit_message>
Write the hand-calculation workbook's formulas as proper maths
</commit_message>
<xml_diff>
--- a/docs/calculation_vs_simulation.xlsx
+++ b/docs/calculation_vs_simulation.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Calc vs Simulation" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Inputs" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Hand calculations" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calc vs Simulation" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hand calculations" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -607,7 +607,23 @@
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>Tank mass m_t</t>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Tank mass m</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>t</t>
+          </r>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
@@ -640,7 +656,23 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>Tank centre-of-mass height above pivot h_t</t>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Tank centre-of-mass height above pivot h</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>t</t>
+          </r>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
@@ -673,12 +705,28 @@
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Tank inertia about pivot I_O</t>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Tank inertia about pivot I</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>O</t>
+          </r>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>kg m^2</t>
+          <t>kg·m²</t>
         </is>
       </c>
       <c r="C7" s="6">
@@ -706,7 +754,23 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>Impulsive water mass m_i</t>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Impulsive water mass m</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>i</t>
+          </r>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
@@ -739,7 +803,23 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>Convective (sloshing) water mass m_c</t>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Convective (sloshing) water mass m</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>c</t>
+          </r>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
@@ -772,7 +852,23 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>Equivalent pendulum length L_p</t>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Equivalent pendulum length L</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>p</t>
+          </r>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
@@ -855,7 +951,7 @@
       </c>
       <c r="F12" s="9" t="inlineStr">
         <is>
-          <t>FFT of the pendulum model's free oscillation (PROJECT_LOG Entry 88)</t>
+          <t>FFT of the pendulum model's free oscillation</t>
         </is>
       </c>
       <c r="G12" s="9" t="inlineStr">
@@ -888,7 +984,7 @@
       </c>
       <c r="F13" s="9" t="inlineStr">
         <is>
-          <t>Peak-to-peak period of the real SPH fluid after a tilt kick (PROJECT_LOG Entry 95)</t>
+          <t>Peak-to-peak period of the real SPH fluid after a tilt kick</t>
         </is>
       </c>
       <c r="G13" s="9" t="inlineStr">
@@ -921,7 +1017,7 @@
       </c>
       <c r="F14" s="9" t="inlineStr">
         <is>
-          <t>Same SPH measurement (Entry 95)</t>
+          <t>Same SPH measurement</t>
         </is>
       </c>
       <c r="G14" s="9" t="inlineStr">
@@ -1278,7 +1374,23 @@
       </c>
       <c r="B8" s="13" t="inlineStr">
         <is>
-          <t>rho_t</t>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+            </rPr>
+            <t>ρ</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>t</t>
+          </r>
         </is>
       </c>
       <c r="C8" s="14" t="n">
@@ -1286,7 +1398,7 @@
       </c>
       <c r="D8" s="13" t="inlineStr">
         <is>
-          <t>kg/m^3</t>
+          <t>kg/m³</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -1328,7 +1440,7 @@
       </c>
       <c r="B10" s="13" t="inlineStr">
         <is>
-          <t>rho</t>
+          <t>ρ</t>
         </is>
       </c>
       <c r="C10" s="14" t="n">
@@ -1336,7 +1448,7 @@
       </c>
       <c r="D10" s="13" t="inlineStr">
         <is>
-          <t>kg/m^3</t>
+          <t>kg/m³</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
@@ -1361,7 +1473,7 @@
       </c>
       <c r="D11" s="13" t="inlineStr">
         <is>
-          <t>m/s^2</t>
+          <t>m/s²</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
@@ -1378,7 +1490,7 @@
       </c>
       <c r="B12" s="13" t="inlineStr">
         <is>
-          <t>mu</t>
+          <t>μ</t>
         </is>
       </c>
       <c r="C12" s="14" t="n">
@@ -1386,7 +1498,7 @@
       </c>
       <c r="D12" s="13" t="inlineStr">
         <is>
-          <t>Pa s</t>
+          <t>Pa·s</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
@@ -1428,7 +1540,23 @@
       </c>
       <c r="B14" s="13" t="inlineStr">
         <is>
-          <t>f_d</t>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+            </rPr>
+            <t>f</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>d</t>
+          </r>
         </is>
       </c>
       <c r="C14" s="14" t="n">
@@ -1453,7 +1581,23 @@
       </c>
       <c r="B15" s="13" t="inlineStr">
         <is>
-          <t>theta_w</t>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+            </rPr>
+            <t>θ</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>w</t>
+          </r>
         </is>
       </c>
       <c r="C15" s="14" t="n">
@@ -1466,7 +1610,7 @@
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>Observed ~9-10 deg in the resonance demo (CLAUDE.md, main.py --fluid-viz-resonance)</t>
+          <t>Observed ~9-10 deg in the resonance demo (main.py --fluid-viz-resonance)</t>
         </is>
       </c>
     </row>
@@ -1478,7 +1622,7 @@
       </c>
       <c r="B16" s="13" t="inlineStr">
         <is>
-          <t>zeta</t>
+          <t>ζ</t>
         </is>
       </c>
       <c r="C16" s="14" t="n">
@@ -1528,7 +1672,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="46" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
@@ -1617,12 +1761,12 @@
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>I about own centre (kg m^2)</t>
+          <t>I about own centre (kg·m²)</t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>I about pivot O (kg m^2)</t>
+          <t>I about pivot O (kg·m²)</t>
         </is>
       </c>
     </row>
@@ -1845,7 +1989,31 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Tank centre of mass height above pivot O, h_t (m)</t>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Tank centre of mass height above pivot O, h</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>t</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve"> = Σ(m·y) / Σm (m)</t>
+          </r>
         </is>
       </c>
       <c r="B11" s="2" t="n"/>
@@ -1863,7 +2031,129 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Inertia about O: I_plate = m(a^2+b^2)/12 + m*(x^2+y^2)  (parallel-axis theorem; rotation axis z through O)</t>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <i val="1"/>
+              <color rgb="00666666"/>
+              <sz val="9"/>
+            </rPr>
+            <t>Plate mass: m = ρ</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <i val="1"/>
+              <color rgb="00666666"/>
+              <sz val="9"/>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>t</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <i val="1"/>
+              <color rgb="00666666"/>
+              <sz val="9"/>
+            </rPr>
+            <t>·a·b·c.   Inertia about O: I</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <i val="1"/>
+              <color rgb="00666666"/>
+              <sz val="9"/>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>O</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <i val="1"/>
+              <color rgb="00666666"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve"> = m(a</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <i val="1"/>
+              <color rgb="00666666"/>
+              <sz val="9"/>
+              <vertAlign val="superscript"/>
+            </rPr>
+            <t>2</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <i val="1"/>
+              <color rgb="00666666"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve"> + b</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <i val="1"/>
+              <color rgb="00666666"/>
+              <sz val="9"/>
+              <vertAlign val="superscript"/>
+            </rPr>
+            <t>2</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <i val="1"/>
+              <color rgb="00666666"/>
+              <sz val="9"/>
+            </rPr>
+            <t>)/12 + m(x</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <i val="1"/>
+              <color rgb="00666666"/>
+              <sz val="9"/>
+              <vertAlign val="superscript"/>
+            </rPr>
+            <t>2</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <i val="1"/>
+              <color rgb="00666666"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve"> + y</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <i val="1"/>
+              <color rgb="00666666"/>
+              <sz val="9"/>
+              <vertAlign val="superscript"/>
+            </rPr>
+            <t>2</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <i val="1"/>
+              <color rgb="00666666"/>
+              <sz val="9"/>
+            </rPr>
+            <t>)  (parallel-axis theorem; rotation axis z through O)</t>
+          </r>
         </is>
       </c>
       <c r="B12" s="2" t="n"/>
@@ -1930,9 +2220,9 @@
           <t>Total water mass m (kg)</t>
         </is>
       </c>
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>rho*L*W*H</t>
+      <c r="B16" s="13" t="inlineStr">
+        <is>
+          <t>m = ρ·L·W·H</t>
         </is>
       </c>
       <c r="C16" s="13">
@@ -1952,9 +2242,9 @@
           <t>Aspect ratio L/H (-)</t>
         </is>
       </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>L/H</t>
+      <c r="B17" s="13" t="inlineStr">
+        <is>
+          <t>L / H</t>
         </is>
       </c>
       <c r="C17" s="13">
@@ -1971,12 +2261,60 @@
     <row r="18">
       <c r="A18" s="13" t="inlineStr">
         <is>
-          <t>Impulsive mass m_i (kg)</t>
-        </is>
-      </c>
-      <c r="B18" s="3" t="inlineStr">
-        <is>
-          <t>tanh(0.866 L/H)/(0.866 L/H) * m</t>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Impulsive mass m</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>i</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve"> (kg)</t>
+          </r>
+        </is>
+      </c>
+      <c r="B18" s="13" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+            </rPr>
+            <t>m</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>i</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve"> = [tanh(0.866·L/H) / (0.866·L/H)]·m</t>
+          </r>
         </is>
       </c>
       <c r="C18" s="13">
@@ -1993,12 +2331,60 @@
     <row r="19">
       <c r="A19" s="13" t="inlineStr">
         <is>
-          <t>Convective mass m_c (kg)</t>
-        </is>
-      </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>0.264 (L/H) tanh(3.16 H/L) * m</t>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Convective mass m</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>c</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve"> (kg)</t>
+          </r>
+        </is>
+      </c>
+      <c r="B19" s="13" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+            </rPr>
+            <t>m</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>c</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve"> = 0.264·(L/H)·tanh(3.16·H/L)·m</t>
+          </r>
         </is>
       </c>
       <c r="C19" s="13">
@@ -2015,12 +2401,60 @@
     <row r="20">
       <c r="A20" s="13" t="inlineStr">
         <is>
-          <t>Impulsive height h_i (m)</t>
-        </is>
-      </c>
-      <c r="B20" s="3" t="inlineStr">
-        <is>
-          <t>(0.5 - 0.09375 L/H) H  [L/H &gt;= 1.333]</t>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Impulsive height h</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>i</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve"> (m)</t>
+          </r>
+        </is>
+      </c>
+      <c r="B20" s="13" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+            </rPr>
+            <t>h</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>i</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve"> = (0.5 − 0.09375·L/H)·H   (for L/H ≥ 1.333)</t>
+          </r>
         </is>
       </c>
       <c r="C20" s="13">
@@ -2037,12 +2471,60 @@
     <row r="21">
       <c r="A21" s="13" t="inlineStr">
         <is>
-          <t>Convective height h_c (m)</t>
-        </is>
-      </c>
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>[1 - (cosh y - 1)/(y sinh y)] H, y = 3.16 H/L</t>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Convective height h</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>c</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve"> (m)</t>
+          </r>
+        </is>
+      </c>
+      <c r="B21" s="13" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+            </rPr>
+            <t>h</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>c</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve"> = [1 − (cosh y − 1) / (y·sinh y)]·H,   y = 3.16·H/L</t>
+          </r>
         </is>
       </c>
       <c r="C21" s="13">
@@ -2059,12 +2541,60 @@
     <row r="22">
       <c r="A22" s="13" t="inlineStr">
         <is>
-          <t>Sloshing natural frequency omega_n (rad/s)</t>
-        </is>
-      </c>
-      <c r="B22" s="3" t="inlineStr">
-        <is>
-          <t>sqrt(3.16 g/L tanh(3.16 H/L))</t>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Sloshing natural frequency ω</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>n</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve"> (rad/s)</t>
+          </r>
+        </is>
+      </c>
+      <c r="B22" s="13" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+            </rPr>
+            <t>ω</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>n</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve"> = √[(3.16·g/L)·tanh(3.16·H/L)]</t>
+          </r>
         </is>
       </c>
       <c r="C22" s="13">
@@ -2081,12 +2611,77 @@
     <row r="23">
       <c r="A23" s="13" t="inlineStr">
         <is>
-          <t>Sloshing natural frequency f_n (Hz)</t>
-        </is>
-      </c>
-      <c r="B23" s="3" t="inlineStr">
-        <is>
-          <t>omega_n / 2 pi</t>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Sloshing natural frequency f</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>n</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve"> (Hz)</t>
+          </r>
+        </is>
+      </c>
+      <c r="B23" s="13" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+            </rPr>
+            <t>f</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>n</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve"> = ω</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>n</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve"> / 2π</t>
+          </r>
         </is>
       </c>
       <c r="C23" s="13">
@@ -2103,12 +2698,78 @@
     <row r="24">
       <c r="A24" s="13" t="inlineStr">
         <is>
-          <t>Equivalent pendulum length L_p (m)</t>
-        </is>
-      </c>
-      <c r="B24" s="3" t="inlineStr">
-        <is>
-          <t>g / omega_n^2</t>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Equivalent pendulum length L</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>p</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve"> (m)</t>
+          </r>
+        </is>
+      </c>
+      <c r="B24" s="13" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+            </rPr>
+            <t>L</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>p</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve"> = g / ω</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>n</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+              <vertAlign val="superscript"/>
+            </rPr>
+            <t>2</t>
+          </r>
         </is>
       </c>
       <c r="C24" s="13">
@@ -2125,10 +2786,55 @@
     <row r="25">
       <c r="A25" s="13" t="inlineStr">
         <is>
-          <t>Modelled mass fraction (m_i+m_c)/m (-)</t>
-        </is>
-      </c>
-      <c r="B25" s="3" t="inlineStr"/>
+          <t>Modelled mass fraction (-)</t>
+        </is>
+      </c>
+      <c r="B25" s="13" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+            </rPr>
+            <t>(m</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>i</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve"> + m</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>c</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+            </rPr>
+            <t>) / m</t>
+          </r>
+        </is>
+      </c>
       <c r="C25" s="13">
         <f>(C18+C19)/C16</f>
         <v/>
@@ -2169,10 +2875,62 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Inner tank length L_in (m)</t>
-        </is>
-      </c>
-      <c r="B28" s="2" t="n"/>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Inner tank length L</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>in</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve"> (m)</t>
+          </r>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+            </rPr>
+            <t>L</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>in</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve"> = L − 2t</t>
+          </r>
+        </is>
+      </c>
       <c r="C28" s="2">
         <f>Inputs!$C$4-2*Inputs!$C$7</f>
         <v/>
@@ -2187,12 +2945,94 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>omega_1 (rad/s)</t>
-        </is>
-      </c>
-      <c r="B29" s="3" t="inlineStr">
-        <is>
-          <t>sqrt(pi g / L_in * tanh(pi H / L_in))</t>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+            </rPr>
+            <t>First-mode frequency ω</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>1</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve"> (rad/s)</t>
+          </r>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+            </rPr>
+            <t>ω</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>1</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve"> = √[(π·g/L</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>in</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+            </rPr>
+            <t>)·tanh(π·H/L</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>in</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+            </rPr>
+            <t>)]</t>
+          </r>
         </is>
       </c>
       <c r="C29" s="2">
@@ -2209,10 +3049,79 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>f_1 (Hz)</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="n"/>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+            </rPr>
+            <t>First-mode frequency f</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>1</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve"> (Hz)</t>
+          </r>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+            </rPr>
+            <t>f</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>1</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve"> = ω</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>1</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve"> / 2π</t>
+          </r>
+        </is>
+      </c>
       <c r="C30" s="2">
         <f>C29/(2*PI())</f>
         <v/>
@@ -2253,10 +3162,71 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Peak tank angular velocity A*2*pi*f_d (rad/s)</t>
-        </is>
-      </c>
-      <c r="B33" s="2" t="n"/>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Peak tank angular velocity Ω</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>max</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve"> (rad/s)</t>
+          </r>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Ω</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>max</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve"> = 2π·A·f</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>d</t>
+          </r>
+        </is>
+      </c>
       <c r="C33" s="2">
         <f>Inputs!$C$13*2*PI()*Inputs!$C$14</f>
         <v/>
@@ -2271,10 +3241,38 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Froude number Fr = theta_dot_max*(L/2)/sqrt(g H)</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="n"/>
+          <t>Froude number Fr (-)</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Fr = Ω</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>max</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+            </rPr>
+            <t>·(L/2) / √(g·H)</t>
+          </r>
+        </is>
+      </c>
       <c r="C34" s="2">
         <f>C33*(Inputs!$C$4/2)/SQRT(Inputs!$C$11*Inputs!$C$9)</f>
         <v/>
@@ -2289,10 +3287,88 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Wave amplitude eta_max = L_p sin(theta_w) (m)</t>
-        </is>
-      </c>
-      <c r="B35" s="2" t="n"/>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Wave amplitude η</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>max</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve"> (m)</t>
+          </r>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+            </rPr>
+            <t>η</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>max</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+            </rPr>
+            <t xml:space="preserve"> = L</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>p</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+            </rPr>
+            <t>·sin θ</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>w</t>
+          </r>
+        </is>
+      </c>
       <c r="C35" s="2">
         <f>C24*SIN(RADIANS(Inputs!$C$15))</f>
         <v/>
@@ -2307,10 +3383,55 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Reynolds number Re = rho*omega_n*eta_max*L/mu</t>
-        </is>
-      </c>
-      <c r="B36" s="2" t="n"/>
+          <t>Reynolds number Re (-)</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Re = ρ·ω</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>n</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+            </rPr>
+            <t>·η</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>max</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="11"/>
+            </rPr>
+            <t>·L / μ</t>
+          </r>
+        </is>
+      </c>
       <c r="C36" s="2">
         <f>Inputs!$C$10*C22*C35*Inputs!$C$4/Inputs!$C$12</f>
         <v/>

</xml_diff>

<commit_message>
Typeset the workbook's formulas as equations
</commit_message>
<xml_diff>
--- a/docs/calculation_vs_simulation.xlsx
+++ b/docs/calculation_vs_simulation.xlsx
@@ -107,7 +107,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -140,6 +140,12 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -229,6 +235,521 @@
     </comment>
   </commentList>
 </comments>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <twoCellAnchor editAs="oneCell">
+    <from>
+      <col>1</col>
+      <colOff>38100</colOff>
+      <row>15</row>
+      <rowOff>28575</rowOff>
+    </from>
+    <to>
+      <col>1</col>
+      <colOff>970788</colOff>
+      <row>15</row>
+      <rowOff>284607</rowOff>
+    </to>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </twoCellAnchor>
+  <twoCellAnchor editAs="oneCell">
+    <from>
+      <col>1</col>
+      <colOff>38100</colOff>
+      <row>16</row>
+      <rowOff>28575</rowOff>
+    </from>
+    <to>
+      <col>1</col>
+      <colOff>248411</colOff>
+      <row>16</row>
+      <rowOff>449198</rowOff>
+    </to>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId2"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </twoCellAnchor>
+  <twoCellAnchor editAs="oneCell">
+    <from>
+      <col>1</col>
+      <colOff>38100</colOff>
+      <row>17</row>
+      <rowOff>28575</rowOff>
+    </from>
+    <to>
+      <col>1</col>
+      <colOff>1866900</colOff>
+      <row>17</row>
+      <rowOff>467487</rowOff>
+    </to>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="3" name="Image 3" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId3"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </twoCellAnchor>
+  <twoCellAnchor editAs="oneCell">
+    <from>
+      <col>1</col>
+      <colOff>38100</colOff>
+      <row>18</row>
+      <rowOff>28575</rowOff>
+    </from>
+    <to>
+      <col>1</col>
+      <colOff>2328672</colOff>
+      <row>18</row>
+      <rowOff>449198</rowOff>
+    </to>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="4" name="Image 4" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId4"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </twoCellAnchor>
+  <twoCellAnchor editAs="oneCell">
+    <from>
+      <col>1</col>
+      <colOff>38100</colOff>
+      <row>19</row>
+      <rowOff>28575</rowOff>
+    </from>
+    <to>
+      <col>1</col>
+      <colOff>3110484</colOff>
+      <row>19</row>
+      <rowOff>449198</rowOff>
+    </to>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="5" name="Image 5" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId5"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </twoCellAnchor>
+  <twoCellAnchor editAs="oneCell">
+    <from>
+      <col>1</col>
+      <colOff>38100</colOff>
+      <row>20</row>
+      <rowOff>28575</rowOff>
+    </from>
+    <to>
+      <col>1</col>
+      <colOff>2785871</colOff>
+      <row>20</row>
+      <rowOff>485775</rowOff>
+    </to>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="6" name="Image 6" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId6"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </twoCellAnchor>
+  <twoCellAnchor editAs="oneCell">
+    <from>
+      <col>1</col>
+      <colOff>38100</colOff>
+      <row>21</row>
+      <rowOff>28575</rowOff>
+    </from>
+    <to>
+      <col>1</col>
+      <colOff>2273808</colOff>
+      <row>21</row>
+      <rowOff>508635</rowOff>
+    </to>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="7" name="Image 7" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId7"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </twoCellAnchor>
+  <twoCellAnchor editAs="oneCell">
+    <from>
+      <col>1</col>
+      <colOff>38100</colOff>
+      <row>22</row>
+      <rowOff>28575</rowOff>
+    </from>
+    <to>
+      <col>1</col>
+      <colOff>646176</colOff>
+      <row>22</row>
+      <rowOff>421767</rowOff>
+    </to>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="8" name="Image 8" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId8"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </twoCellAnchor>
+  <twoCellAnchor editAs="oneCell">
+    <from>
+      <col>1</col>
+      <colOff>38100</colOff>
+      <row>23</row>
+      <rowOff>28575</rowOff>
+    </from>
+    <to>
+      <col>1</col>
+      <colOff>701040</colOff>
+      <row>23</row>
+      <rowOff>490346</rowOff>
+    </to>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="9" name="Image 9" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId9"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </twoCellAnchor>
+  <twoCellAnchor editAs="oneCell">
+    <from>
+      <col>1</col>
+      <colOff>38100</colOff>
+      <row>24</row>
+      <rowOff>28575</rowOff>
+    </from>
+    <to>
+      <col>1</col>
+      <colOff>714755</colOff>
+      <row>24</row>
+      <rowOff>430910</rowOff>
+    </to>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="10" name="Image 10" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId10"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </twoCellAnchor>
+  <twoCellAnchor editAs="oneCell">
+    <from>
+      <col>1</col>
+      <colOff>38100</colOff>
+      <row>27</row>
+      <rowOff>28575</rowOff>
+    </from>
+    <to>
+      <col>1</col>
+      <colOff>915924</colOff>
+      <row>27</row>
+      <rowOff>284607</rowOff>
+    </to>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="11" name="Image 11" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId11"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </twoCellAnchor>
+  <twoCellAnchor editAs="oneCell">
+    <from>
+      <col>1</col>
+      <colOff>38100</colOff>
+      <row>28</row>
+      <rowOff>28575</rowOff>
+    </from>
+    <to>
+      <col>1</col>
+      <colOff>1757172</colOff>
+      <row>28</row>
+      <rowOff>526923</rowOff>
+    </to>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="12" name="Image 12" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId12"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </twoCellAnchor>
+  <twoCellAnchor editAs="oneCell">
+    <from>
+      <col>1</col>
+      <colOff>38100</colOff>
+      <row>29</row>
+      <rowOff>28575</rowOff>
+    </from>
+    <to>
+      <col>1</col>
+      <colOff>646176</colOff>
+      <row>29</row>
+      <rowOff>421767</rowOff>
+    </to>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="13" name="Image 13" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId13"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </twoCellAnchor>
+  <twoCellAnchor editAs="oneCell">
+    <from>
+      <col>1</col>
+      <colOff>38100</colOff>
+      <row>32</row>
+      <rowOff>28575</rowOff>
+    </from>
+    <to>
+      <col>1</col>
+      <colOff>1121664</colOff>
+      <row>32</row>
+      <rowOff>284607</rowOff>
+    </to>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="14" name="Image 14" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId14"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </twoCellAnchor>
+  <twoCellAnchor editAs="oneCell">
+    <from>
+      <col>1</col>
+      <colOff>38100</colOff>
+      <row>33</row>
+      <rowOff>28575</rowOff>
+    </from>
+    <to>
+      <col>1</col>
+      <colOff>1199388</colOff>
+      <row>33</row>
+      <rowOff>531495</rowOff>
+    </to>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="15" name="Image 15" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId15"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </twoCellAnchor>
+  <twoCellAnchor editAs="oneCell">
+    <from>
+      <col>1</col>
+      <colOff>38100</colOff>
+      <row>34</row>
+      <rowOff>28575</rowOff>
+    </from>
+    <to>
+      <col>1</col>
+      <colOff>1245108</colOff>
+      <row>34</row>
+      <rowOff>293751</rowOff>
+    </to>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="16" name="Image 16" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId16"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </twoCellAnchor>
+  <twoCellAnchor editAs="oneCell">
+    <from>
+      <col>1</col>
+      <colOff>38100</colOff>
+      <row>35</row>
+      <rowOff>28575</rowOff>
+    </from>
+    <to>
+      <col>1</col>
+      <colOff>1309116</colOff>
+      <row>35</row>
+      <rowOff>481202</rowOff>
+    </to>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="17" name="Image 17" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId17"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </twoCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1682,7 +2203,7 @@
     <col width="18" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Hand calculations (every number below is an Excel formula)</t>
@@ -1697,7 +2218,7 @@
       <c r="H1" s="2" t="n"/>
       <c r="I1" s="2" t="n"/>
     </row>
-    <row r="2">
+    <row r="2" ht="15" customHeight="1">
       <c r="A2" s="2" t="n"/>
       <c r="B2" s="2" t="n"/>
       <c r="C2" s="2" t="n"/>
@@ -1708,7 +2229,7 @@
       <c r="H2" s="2" t="n"/>
       <c r="I2" s="2" t="n"/>
     </row>
-    <row r="3">
+    <row r="3" ht="15" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>1. Tank mass and inertia from its five acrylic plates</t>
@@ -1723,7 +2244,7 @@
       <c r="H3" s="2" t="n"/>
       <c r="I3" s="2" t="n"/>
     </row>
-    <row r="4">
+    <row r="4" ht="30" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Plate</t>
@@ -1770,7 +2291,7 @@
         </is>
       </c>
     </row>
-    <row r="5">
+    <row r="5" ht="15" customHeight="1">
       <c r="A5" s="13" t="inlineStr">
         <is>
           <t>Base</t>
@@ -1809,7 +2330,7 @@
         <v/>
       </c>
     </row>
-    <row r="6">
+    <row r="6" ht="15" customHeight="1">
       <c r="A6" s="13" t="inlineStr">
         <is>
           <t>Side wall (+z)</t>
@@ -1848,7 +2369,7 @@
         <v/>
       </c>
     </row>
-    <row r="7">
+    <row r="7" ht="15" customHeight="1">
       <c r="A7" s="13" t="inlineStr">
         <is>
           <t>Side wall (-z)</t>
@@ -1887,7 +2408,7 @@
         <v/>
       </c>
     </row>
-    <row r="8">
+    <row r="8" ht="15" customHeight="1">
       <c r="A8" s="13" t="inlineStr">
         <is>
           <t>End wall (+x)</t>
@@ -1926,7 +2447,7 @@
         <v/>
       </c>
     </row>
-    <row r="9">
+    <row r="9" ht="15" customHeight="1">
       <c r="A9" s="13" t="inlineStr">
         <is>
           <t>End wall (-x)</t>
@@ -1965,7 +2486,7 @@
         <v/>
       </c>
     </row>
-    <row r="10">
+    <row r="10" ht="15" customHeight="1">
       <c r="A10" s="12" t="inlineStr">
         <is>
           <t>Total</t>
@@ -1986,7 +2507,7 @@
         <v/>
       </c>
     </row>
-    <row r="11">
+    <row r="11" ht="15" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
           <r>
@@ -2028,7 +2549,7 @@
       <c r="H11" s="2" t="n"/>
       <c r="I11" s="2" t="n"/>
     </row>
-    <row r="12">
+    <row r="12" ht="15" customHeight="1">
       <c r="A12" s="3" t="inlineStr">
         <is>
           <r>
@@ -2165,7 +2686,7 @@
       <c r="H12" s="2" t="n"/>
       <c r="I12" s="2" t="n"/>
     </row>
-    <row r="13">
+    <row r="13" ht="15" customHeight="1">
       <c r="A13" s="2" t="n"/>
       <c r="B13" s="2" t="n"/>
       <c r="C13" s="2" t="n"/>
@@ -2176,7 +2697,7 @@
       <c r="H13" s="2" t="n"/>
       <c r="I13" s="2" t="n"/>
     </row>
-    <row r="14">
+    <row r="14" ht="15" customHeight="1">
       <c r="A14" s="12" t="inlineStr">
         <is>
           <t>2. Housner (1963) / ACI 350.3-06 equivalent model of the water</t>
@@ -2191,7 +2712,7 @@
       <c r="H14" s="2" t="n"/>
       <c r="I14" s="2" t="n"/>
     </row>
-    <row r="15">
+    <row r="15" ht="15" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
         <is>
           <t>Quantity</t>
@@ -2214,18 +2735,14 @@
       <c r="H15" s="2" t="n"/>
       <c r="I15" s="2" t="n"/>
     </row>
-    <row r="16">
-      <c r="A16" s="13" t="inlineStr">
+    <row r="16" ht="26.16" customHeight="1">
+      <c r="A16" s="16" t="inlineStr">
         <is>
           <t>Total water mass m (kg)</t>
         </is>
       </c>
-      <c r="B16" s="13" t="inlineStr">
-        <is>
-          <t>m = ρ·L·W·H</t>
-        </is>
-      </c>
-      <c r="C16" s="13">
+      <c r="B16" s="13" t="n"/>
+      <c r="C16" s="16">
         <f>Inputs!$C$10*Inputs!$C$4*Inputs!$C$5*Inputs!$C$9</f>
         <v/>
       </c>
@@ -2236,18 +2753,14 @@
       <c r="H16" s="2" t="n"/>
       <c r="I16" s="2" t="n"/>
     </row>
-    <row r="17">
-      <c r="A17" s="13" t="inlineStr">
+    <row r="17" ht="39.12" customHeight="1">
+      <c r="A17" s="16" t="inlineStr">
         <is>
           <t>Aspect ratio L/H (-)</t>
         </is>
       </c>
-      <c r="B17" s="13" t="inlineStr">
-        <is>
-          <t>L / H</t>
-        </is>
-      </c>
-      <c r="C17" s="13">
+      <c r="B17" s="13" t="n"/>
+      <c r="C17" s="16">
         <f>Inputs!$C$4/Inputs!$C$9</f>
         <v/>
       </c>
@@ -2258,8 +2771,8 @@
       <c r="H17" s="2" t="n"/>
       <c r="I17" s="2" t="n"/>
     </row>
-    <row r="18">
-      <c r="A18" s="13" t="inlineStr">
+    <row r="18" ht="40.56" customHeight="1">
+      <c r="A18" s="16" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2288,36 +2801,8 @@
           </r>
         </is>
       </c>
-      <c r="B18" s="13" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="00000000"/>
-              <sz val="11"/>
-            </rPr>
-            <t>m</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="00000000"/>
-              <sz val="11"/>
-              <vertAlign val="subscript"/>
-            </rPr>
-            <t>i</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="00000000"/>
-              <sz val="11"/>
-            </rPr>
-            <t xml:space="preserve"> = [tanh(0.866·L/H) / (0.866·L/H)]·m</t>
-          </r>
-        </is>
-      </c>
-      <c r="C18" s="13">
+      <c r="B18" s="13" t="n"/>
+      <c r="C18" s="16">
         <f>TANH(0.866*C17)/(0.866*C17)*C16</f>
         <v/>
       </c>
@@ -2328,8 +2813,8 @@
       <c r="H18" s="2" t="n"/>
       <c r="I18" s="2" t="n"/>
     </row>
-    <row r="19">
-      <c r="A19" s="13" t="inlineStr">
+    <row r="19" ht="39.12" customHeight="1">
+      <c r="A19" s="16" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2358,36 +2843,8 @@
           </r>
         </is>
       </c>
-      <c r="B19" s="13" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="00000000"/>
-              <sz val="11"/>
-            </rPr>
-            <t>m</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="00000000"/>
-              <sz val="11"/>
-              <vertAlign val="subscript"/>
-            </rPr>
-            <t>c</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="00000000"/>
-              <sz val="11"/>
-            </rPr>
-            <t xml:space="preserve"> = 0.264·(L/H)·tanh(3.16·H/L)·m</t>
-          </r>
-        </is>
-      </c>
-      <c r="C19" s="13">
+      <c r="B19" s="13" t="n"/>
+      <c r="C19" s="16">
         <f>0.264*C17*TANH(3.16*Inputs!$C$9/Inputs!$C$4)*C16</f>
         <v/>
       </c>
@@ -2398,8 +2855,8 @@
       <c r="H19" s="2" t="n"/>
       <c r="I19" s="2" t="n"/>
     </row>
-    <row r="20">
-      <c r="A20" s="13" t="inlineStr">
+    <row r="20" ht="39.12" customHeight="1">
+      <c r="A20" s="16" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2428,36 +2885,8 @@
           </r>
         </is>
       </c>
-      <c r="B20" s="13" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="00000000"/>
-              <sz val="11"/>
-            </rPr>
-            <t>h</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="00000000"/>
-              <sz val="11"/>
-              <vertAlign val="subscript"/>
-            </rPr>
-            <t>i</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="00000000"/>
-              <sz val="11"/>
-            </rPr>
-            <t xml:space="preserve"> = (0.5 − 0.09375·L/H)·H   (for L/H ≥ 1.333)</t>
-          </r>
-        </is>
-      </c>
-      <c r="C20" s="13">
+      <c r="B20" s="13" t="n"/>
+      <c r="C20" s="16">
         <f>IF(C17&gt;=1.333,0.5-0.09375*C17,0.375)*Inputs!$C$9</f>
         <v/>
       </c>
@@ -2468,8 +2897,8 @@
       <c r="H20" s="2" t="n"/>
       <c r="I20" s="2" t="n"/>
     </row>
-    <row r="21">
-      <c r="A21" s="13" t="inlineStr">
+    <row r="21" ht="42" customHeight="1">
+      <c r="A21" s="16" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2498,36 +2927,8 @@
           </r>
         </is>
       </c>
-      <c r="B21" s="13" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="00000000"/>
-              <sz val="11"/>
-            </rPr>
-            <t>h</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="00000000"/>
-              <sz val="11"/>
-              <vertAlign val="subscript"/>
-            </rPr>
-            <t>c</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="00000000"/>
-              <sz val="11"/>
-            </rPr>
-            <t xml:space="preserve"> = [1 − (cosh y − 1) / (y·sinh y)]·H,   y = 3.16·H/L</t>
-          </r>
-        </is>
-      </c>
-      <c r="C21" s="13">
+      <c r="B21" s="13" t="n"/>
+      <c r="C21" s="16">
         <f>(1-(COSH(3.16*Inputs!$C$9/Inputs!$C$4)-1)/(3.16*Inputs!$C$9/Inputs!$C$4*SINH(3.16*Inputs!$C$9/Inputs!$C$4)))*Inputs!$C$9</f>
         <v/>
       </c>
@@ -2538,8 +2939,8 @@
       <c r="H21" s="2" t="n"/>
       <c r="I21" s="2" t="n"/>
     </row>
-    <row r="22">
-      <c r="A22" s="13" t="inlineStr">
+    <row r="22" ht="43.8" customHeight="1">
+      <c r="A22" s="16" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2568,36 +2969,8 @@
           </r>
         </is>
       </c>
-      <c r="B22" s="13" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="00000000"/>
-              <sz val="11"/>
-            </rPr>
-            <t>ω</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="00000000"/>
-              <sz val="11"/>
-              <vertAlign val="subscript"/>
-            </rPr>
-            <t>n</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="00000000"/>
-              <sz val="11"/>
-            </rPr>
-            <t xml:space="preserve"> = √[(3.16·g/L)·tanh(3.16·H/L)]</t>
-          </r>
-        </is>
-      </c>
-      <c r="C22" s="13">
+      <c r="B22" s="13" t="n"/>
+      <c r="C22" s="16">
         <f>SQRT(3.16*Inputs!$C$11/Inputs!$C$4*TANH(3.16*Inputs!$C$9/Inputs!$C$4))</f>
         <v/>
       </c>
@@ -2608,8 +2981,8 @@
       <c r="H22" s="2" t="n"/>
       <c r="I22" s="2" t="n"/>
     </row>
-    <row r="23">
-      <c r="A23" s="13" t="inlineStr">
+    <row r="23" ht="36.96" customHeight="1">
+      <c r="A23" s="16" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2638,53 +3011,8 @@
           </r>
         </is>
       </c>
-      <c r="B23" s="13" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="00000000"/>
-              <sz val="11"/>
-            </rPr>
-            <t>f</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="00000000"/>
-              <sz val="11"/>
-              <vertAlign val="subscript"/>
-            </rPr>
-            <t>n</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="00000000"/>
-              <sz val="11"/>
-            </rPr>
-            <t xml:space="preserve"> = ω</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="00000000"/>
-              <sz val="11"/>
-              <vertAlign val="subscript"/>
-            </rPr>
-            <t>n</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="00000000"/>
-              <sz val="11"/>
-            </rPr>
-            <t xml:space="preserve"> / 2π</t>
-          </r>
-        </is>
-      </c>
-      <c r="C23" s="13">
+      <c r="B23" s="13" t="n"/>
+      <c r="C23" s="16">
         <f>C22/(2*PI())</f>
         <v/>
       </c>
@@ -2695,8 +3023,8 @@
       <c r="H23" s="2" t="n"/>
       <c r="I23" s="2" t="n"/>
     </row>
-    <row r="24">
-      <c r="A24" s="13" t="inlineStr">
+    <row r="24" ht="42.36" customHeight="1">
+      <c r="A24" s="16" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2725,54 +3053,8 @@
           </r>
         </is>
       </c>
-      <c r="B24" s="13" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="00000000"/>
-              <sz val="11"/>
-            </rPr>
-            <t>L</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="00000000"/>
-              <sz val="11"/>
-              <vertAlign val="subscript"/>
-            </rPr>
-            <t>p</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="00000000"/>
-              <sz val="11"/>
-            </rPr>
-            <t xml:space="preserve"> = g / ω</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="00000000"/>
-              <sz val="11"/>
-              <vertAlign val="subscript"/>
-            </rPr>
-            <t>n</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="00000000"/>
-              <sz val="11"/>
-              <vertAlign val="superscript"/>
-            </rPr>
-            <t>2</t>
-          </r>
-        </is>
-      </c>
-      <c r="C24" s="13">
+      <c r="B24" s="13" t="n"/>
+      <c r="C24" s="16">
         <f>Inputs!$C$11/C22^2</f>
         <v/>
       </c>
@@ -2783,59 +3065,14 @@
       <c r="H24" s="2" t="n"/>
       <c r="I24" s="2" t="n"/>
     </row>
-    <row r="25">
-      <c r="A25" s="13" t="inlineStr">
+    <row r="25" ht="37.67999999999999" customHeight="1">
+      <c r="A25" s="16" t="inlineStr">
         <is>
           <t>Modelled mass fraction (-)</t>
         </is>
       </c>
-      <c r="B25" s="13" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="00000000"/>
-              <sz val="11"/>
-            </rPr>
-            <t>(m</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="00000000"/>
-              <sz val="11"/>
-              <vertAlign val="subscript"/>
-            </rPr>
-            <t>i</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="00000000"/>
-              <sz val="11"/>
-            </rPr>
-            <t xml:space="preserve"> + m</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="00000000"/>
-              <sz val="11"/>
-              <vertAlign val="subscript"/>
-            </rPr>
-            <t>c</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="00000000"/>
-              <sz val="11"/>
-            </rPr>
-            <t>) / m</t>
-          </r>
-        </is>
-      </c>
-      <c r="C25" s="13">
+      <c r="B25" s="13" t="n"/>
+      <c r="C25" s="16">
         <f>(C18+C19)/C16</f>
         <v/>
       </c>
@@ -2846,7 +3083,7 @@
       <c r="H25" s="2" t="n"/>
       <c r="I25" s="2" t="n"/>
     </row>
-    <row r="26">
+    <row r="26" ht="15" customHeight="1">
       <c r="A26" s="2" t="n"/>
       <c r="B26" s="2" t="n"/>
       <c r="C26" s="2" t="n"/>
@@ -2857,7 +3094,7 @@
       <c r="H26" s="2" t="n"/>
       <c r="I26" s="2" t="n"/>
     </row>
-    <row r="27">
+    <row r="27" ht="15" customHeight="1">
       <c r="A27" s="12" t="inlineStr">
         <is>
           <t>3. Exact linear potential-flow sloshing frequency (alternative analytical check)</t>
@@ -2872,8 +3109,8 @@
       <c r="H27" s="2" t="n"/>
       <c r="I27" s="2" t="n"/>
     </row>
-    <row r="28">
-      <c r="A28" s="2" t="inlineStr">
+    <row r="28" ht="26.16" customHeight="1">
+      <c r="A28" s="17" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2902,36 +3139,8 @@
           </r>
         </is>
       </c>
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="00000000"/>
-              <sz val="11"/>
-            </rPr>
-            <t>L</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="00000000"/>
-              <sz val="11"/>
-              <vertAlign val="subscript"/>
-            </rPr>
-            <t>in</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="00000000"/>
-              <sz val="11"/>
-            </rPr>
-            <t xml:space="preserve"> = L − 2t</t>
-          </r>
-        </is>
-      </c>
-      <c r="C28" s="2">
+      <c r="B28" s="2" t="n"/>
+      <c r="C28" s="17">
         <f>Inputs!$C$4-2*Inputs!$C$7</f>
         <v/>
       </c>
@@ -2942,8 +3151,8 @@
       <c r="H28" s="2" t="n"/>
       <c r="I28" s="2" t="n"/>
     </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr">
+    <row r="29" ht="45.24" customHeight="1">
+      <c r="A29" s="17" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2972,70 +3181,8 @@
           </r>
         </is>
       </c>
-      <c r="B29" s="2" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="00000000"/>
-              <sz val="11"/>
-            </rPr>
-            <t>ω</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="00000000"/>
-              <sz val="11"/>
-              <vertAlign val="subscript"/>
-            </rPr>
-            <t>1</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="00000000"/>
-              <sz val="11"/>
-            </rPr>
-            <t xml:space="preserve"> = √[(π·g/L</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="00000000"/>
-              <sz val="11"/>
-              <vertAlign val="subscript"/>
-            </rPr>
-            <t>in</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="00000000"/>
-              <sz val="11"/>
-            </rPr>
-            <t>)·tanh(π·H/L</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="00000000"/>
-              <sz val="11"/>
-              <vertAlign val="subscript"/>
-            </rPr>
-            <t>in</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="00000000"/>
-              <sz val="11"/>
-            </rPr>
-            <t>)]</t>
-          </r>
-        </is>
-      </c>
-      <c r="C29" s="2">
+      <c r="B29" s="2" t="n"/>
+      <c r="C29" s="17">
         <f>SQRT(PI()*Inputs!$C$11/C28*TANH(PI()*Inputs!$C$9/C28))</f>
         <v/>
       </c>
@@ -3046,8 +3193,8 @@
       <c r="H29" s="2" t="n"/>
       <c r="I29" s="2" t="n"/>
     </row>
-    <row r="30">
-      <c r="A30" s="2" t="inlineStr">
+    <row r="30" ht="36.96" customHeight="1">
+      <c r="A30" s="17" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3076,53 +3223,8 @@
           </r>
         </is>
       </c>
-      <c r="B30" s="2" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="00000000"/>
-              <sz val="11"/>
-            </rPr>
-            <t>f</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="00000000"/>
-              <sz val="11"/>
-              <vertAlign val="subscript"/>
-            </rPr>
-            <t>1</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="00000000"/>
-              <sz val="11"/>
-            </rPr>
-            <t xml:space="preserve"> = ω</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="00000000"/>
-              <sz val="11"/>
-              <vertAlign val="subscript"/>
-            </rPr>
-            <t>1</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="00000000"/>
-              <sz val="11"/>
-            </rPr>
-            <t xml:space="preserve"> / 2π</t>
-          </r>
-        </is>
-      </c>
-      <c r="C30" s="2">
+      <c r="B30" s="2" t="n"/>
+      <c r="C30" s="17">
         <f>C29/(2*PI())</f>
         <v/>
       </c>
@@ -3133,7 +3235,7 @@
       <c r="H30" s="2" t="n"/>
       <c r="I30" s="2" t="n"/>
     </row>
-    <row r="31">
+    <row r="31" ht="15" customHeight="1">
       <c r="A31" s="2" t="n"/>
       <c r="B31" s="2" t="n"/>
       <c r="C31" s="2" t="n"/>
@@ -3144,7 +3246,7 @@
       <c r="H31" s="2" t="n"/>
       <c r="I31" s="2" t="n"/>
     </row>
-    <row r="32">
+    <row r="32" ht="15" customHeight="1">
       <c r="A32" s="12" t="inlineStr">
         <is>
           <t>4. Non-dimensional numbers (flow regime)</t>
@@ -3159,8 +3261,8 @@
       <c r="H32" s="2" t="n"/>
       <c r="I32" s="2" t="n"/>
     </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr">
+    <row r="33" ht="26.16" customHeight="1">
+      <c r="A33" s="17" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3189,45 +3291,8 @@
           </r>
         </is>
       </c>
-      <c r="B33" s="2" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="00000000"/>
-              <sz val="11"/>
-            </rPr>
-            <t>Ω</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="00000000"/>
-              <sz val="11"/>
-              <vertAlign val="subscript"/>
-            </rPr>
-            <t>max</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="00000000"/>
-              <sz val="11"/>
-            </rPr>
-            <t xml:space="preserve"> = 2π·A·f</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="00000000"/>
-              <sz val="11"/>
-              <vertAlign val="subscript"/>
-            </rPr>
-            <t>d</t>
-          </r>
-        </is>
-      </c>
-      <c r="C33" s="2">
+      <c r="B33" s="2" t="n"/>
+      <c r="C33" s="17">
         <f>Inputs!$C$13*2*PI()*Inputs!$C$14</f>
         <v/>
       </c>
@@ -3238,42 +3303,14 @@
       <c r="H33" s="2" t="n"/>
       <c r="I33" s="2" t="n"/>
     </row>
-    <row r="34">
-      <c r="A34" s="2" t="inlineStr">
+    <row r="34" ht="45.59999999999999" customHeight="1">
+      <c r="A34" s="17" t="inlineStr">
         <is>
           <t>Froude number Fr (-)</t>
         </is>
       </c>
-      <c r="B34" s="2" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="00000000"/>
-              <sz val="11"/>
-            </rPr>
-            <t>Fr = Ω</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="00000000"/>
-              <sz val="11"/>
-              <vertAlign val="subscript"/>
-            </rPr>
-            <t>max</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="00000000"/>
-              <sz val="11"/>
-            </rPr>
-            <t>·(L/2) / √(g·H)</t>
-          </r>
-        </is>
-      </c>
-      <c r="C34" s="2">
+      <c r="B34" s="2" t="n"/>
+      <c r="C34" s="17">
         <f>C33*(Inputs!$C$4/2)/SQRT(Inputs!$C$11*Inputs!$C$9)</f>
         <v/>
       </c>
@@ -3284,8 +3321,8 @@
       <c r="H34" s="2" t="n"/>
       <c r="I34" s="2" t="n"/>
     </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr">
+    <row r="35" ht="26.88" customHeight="1">
+      <c r="A35" s="17" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3314,62 +3351,8 @@
           </r>
         </is>
       </c>
-      <c r="B35" s="2" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="00000000"/>
-              <sz val="11"/>
-            </rPr>
-            <t>η</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="00000000"/>
-              <sz val="11"/>
-              <vertAlign val="subscript"/>
-            </rPr>
-            <t>max</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="00000000"/>
-              <sz val="11"/>
-            </rPr>
-            <t xml:space="preserve"> = L</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="00000000"/>
-              <sz val="11"/>
-              <vertAlign val="subscript"/>
-            </rPr>
-            <t>p</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="00000000"/>
-              <sz val="11"/>
-            </rPr>
-            <t>·sin θ</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="00000000"/>
-              <sz val="11"/>
-              <vertAlign val="subscript"/>
-            </rPr>
-            <t>w</t>
-          </r>
-        </is>
-      </c>
-      <c r="C35" s="2">
+      <c r="B35" s="2" t="n"/>
+      <c r="C35" s="17">
         <f>C24*SIN(RADIANS(Inputs!$C$15))</f>
         <v/>
       </c>
@@ -3380,59 +3363,14 @@
       <c r="H35" s="2" t="n"/>
       <c r="I35" s="2" t="n"/>
     </row>
-    <row r="36">
-      <c r="A36" s="2" t="inlineStr">
+    <row r="36" ht="41.64" customHeight="1">
+      <c r="A36" s="17" t="inlineStr">
         <is>
           <t>Reynolds number Re (-)</t>
         </is>
       </c>
-      <c r="B36" s="2" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="00000000"/>
-              <sz val="11"/>
-            </rPr>
-            <t>Re = ρ·ω</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="00000000"/>
-              <sz val="11"/>
-              <vertAlign val="subscript"/>
-            </rPr>
-            <t>n</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="00000000"/>
-              <sz val="11"/>
-            </rPr>
-            <t>·η</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="00000000"/>
-              <sz val="11"/>
-              <vertAlign val="subscript"/>
-            </rPr>
-            <t>max</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="00000000"/>
-              <sz val="11"/>
-            </rPr>
-            <t>·L / μ</t>
-          </r>
-        </is>
-      </c>
-      <c r="C36" s="2">
+      <c r="B36" s="2" t="n"/>
+      <c r="C36" s="17">
         <f>Inputs!$C$10*C22*C35*Inputs!$C$4/Inputs!$C$12</f>
         <v/>
       </c>
@@ -3443,7 +3381,7 @@
       <c r="H36" s="2" t="n"/>
       <c r="I36" s="2" t="n"/>
     </row>
-    <row r="37">
+    <row r="37" ht="15" customHeight="1">
       <c r="A37" s="3" t="inlineStr">
         <is>
           <t>Fr &lt;&lt; 0.2 means small, smooth (linear) sloshing; Re ~1e4-1e5 is typical of lab-scale water sloshing.</t>
@@ -3460,5 +3398,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>